<commit_message>
21/09/2026 update (calculation processes)
</commit_message>
<xml_diff>
--- a/GHG_Calculation/output/anaerobic_summary_by_country.xlsx
+++ b/GHG_Calculation/output/anaerobic_summary_by_country.xlsx
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>4397</v>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="D2" t="n">
-        <v>43.8</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>685370</v>
+        <v>99239738</v>
       </c>
       <c r="F2" t="n">
-        <v>589820</v>
+        <v>81633783</v>
       </c>
       <c r="G2" t="n">
-        <v>86.09999999999999</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="3">
@@ -500,544 +500,544 @@
         <v>1885</v>
       </c>
       <c r="C3" t="n">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="D3" t="n">
-        <v>18</v>
+        <v>18.6</v>
       </c>
       <c r="E3" t="n">
         <v>70361227</v>
       </c>
       <c r="F3" t="n">
-        <v>51650375</v>
+        <v>52036338</v>
       </c>
       <c r="G3" t="n">
-        <v>73.40000000000001</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4397</v>
+        <v>32</v>
       </c>
       <c r="C4" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>2.1</v>
+        <v>21.9</v>
       </c>
       <c r="E4" t="n">
-        <v>99239738</v>
+        <v>685370</v>
       </c>
       <c r="F4" t="n">
-        <v>70227246</v>
+        <v>466200</v>
       </c>
       <c r="G4" t="n">
-        <v>70.8</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>323</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>122</v>
       </c>
       <c r="D5" t="n">
-        <v>13.7</v>
+        <v>37.8</v>
       </c>
       <c r="E5" t="n">
-        <v>1280340</v>
+        <v>15079880</v>
       </c>
       <c r="F5" t="n">
-        <v>897114</v>
+        <v>10166604</v>
       </c>
       <c r="G5" t="n">
-        <v>70.09999999999999</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>517</v>
+        <v>2818</v>
       </c>
       <c r="C6" t="n">
-        <v>68</v>
+        <v>218</v>
       </c>
       <c r="D6" t="n">
-        <v>13.2</v>
+        <v>7.7</v>
       </c>
       <c r="E6" t="n">
-        <v>12215992</v>
+        <v>71701510</v>
       </c>
       <c r="F6" t="n">
-        <v>7796765</v>
+        <v>44755418</v>
       </c>
       <c r="G6" t="n">
-        <v>63.8</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>261</v>
+        <v>2198</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>211</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>9.6</v>
       </c>
       <c r="E7" t="n">
-        <v>9988743</v>
+        <v>70746391</v>
       </c>
       <c r="F7" t="n">
-        <v>6106399</v>
+        <v>41851716</v>
       </c>
       <c r="G7" t="n">
-        <v>61.1</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>771</v>
+        <v>261</v>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="D8" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
       <c r="E8" t="n">
-        <v>7833065</v>
+        <v>9988743</v>
       </c>
       <c r="F8" t="n">
-        <v>4730983</v>
+        <v>5853442</v>
       </c>
       <c r="G8" t="n">
-        <v>60.4</v>
+        <v>58.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2198</v>
+        <v>517</v>
       </c>
       <c r="C9" t="n">
-        <v>250</v>
+        <v>53</v>
       </c>
       <c r="D9" t="n">
-        <v>11.4</v>
+        <v>10.3</v>
       </c>
       <c r="E9" t="n">
-        <v>70746391</v>
+        <v>12215992</v>
       </c>
       <c r="F9" t="n">
-        <v>41852367</v>
+        <v>7013140</v>
       </c>
       <c r="G9" t="n">
-        <v>59.2</v>
+        <v>57.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Cyprus</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>4.2</v>
+        <v>16.7</v>
       </c>
       <c r="E10" t="n">
-        <v>1462612</v>
+        <v>946924</v>
       </c>
       <c r="F10" t="n">
-        <v>824822</v>
+        <v>519949</v>
       </c>
       <c r="G10" t="n">
-        <v>56.4</v>
+        <v>54.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>631</v>
+        <v>771</v>
       </c>
       <c r="C11" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>5.3</v>
       </c>
       <c r="E11" t="n">
-        <v>21988660</v>
+        <v>7833065</v>
       </c>
       <c r="F11" t="n">
-        <v>12180517</v>
+        <v>4194865</v>
       </c>
       <c r="G11" t="n">
-        <v>55.4</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2818</v>
+        <v>22303</v>
       </c>
       <c r="C12" t="n">
-        <v>225</v>
+        <v>297</v>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>1.3</v>
       </c>
       <c r="E12" t="n">
-        <v>71701510</v>
+        <v>78634473</v>
       </c>
       <c r="F12" t="n">
-        <v>37774749</v>
+        <v>40276033</v>
       </c>
       <c r="G12" t="n">
-        <v>52.7</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>830</v>
+        <v>1051</v>
       </c>
       <c r="C13" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>1.3</v>
       </c>
       <c r="E13" t="n">
-        <v>10573962</v>
+        <v>6287249</v>
       </c>
       <c r="F13" t="n">
-        <v>5106635</v>
+        <v>3117900</v>
       </c>
       <c r="G13" t="n">
-        <v>48.3</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>610</v>
+        <v>631</v>
       </c>
       <c r="C14" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="D14" t="n">
-        <v>4.4</v>
+        <v>8.1</v>
       </c>
       <c r="E14" t="n">
-        <v>10380012</v>
+        <v>21988660</v>
       </c>
       <c r="F14" t="n">
-        <v>4966674</v>
+        <v>10571732</v>
       </c>
       <c r="G14" t="n">
-        <v>47.8</v>
+        <v>48.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>120</v>
+        <v>51</v>
       </c>
       <c r="C15" t="n">
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>6.7</v>
+        <v>15.7</v>
       </c>
       <c r="E15" t="n">
-        <v>5836054</v>
+        <v>1280340</v>
       </c>
       <c r="F15" t="n">
-        <v>2784573</v>
+        <v>587591</v>
       </c>
       <c r="G15" t="n">
-        <v>47.7</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>22303</v>
+        <v>117</v>
       </c>
       <c r="C16" t="n">
-        <v>238</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>1.1</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>78634473</v>
+        <v>1652034</v>
       </c>
       <c r="F16" t="n">
-        <v>36723565</v>
+        <v>755300</v>
       </c>
       <c r="G16" t="n">
-        <v>46.7</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>402</v>
+        <v>120</v>
       </c>
       <c r="C17" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>10.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>7482609</v>
+        <v>5836054</v>
       </c>
       <c r="F17" t="n">
-        <v>3114048</v>
+        <v>2645212</v>
       </c>
       <c r="G17" t="n">
-        <v>41.6</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1710</v>
+        <v>402</v>
       </c>
       <c r="C18" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="D18" t="n">
-        <v>5.7</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>37638384</v>
+        <v>7482609</v>
       </c>
       <c r="F18" t="n">
-        <v>15556434</v>
+        <v>3209500</v>
       </c>
       <c r="G18" t="n">
-        <v>41.3</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Cyprus</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>18</v>
+        <v>830</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="D19" t="n">
-        <v>11.1</v>
+        <v>3.1</v>
       </c>
       <c r="E19" t="n">
-        <v>946924</v>
+        <v>10573962</v>
       </c>
       <c r="F19" t="n">
-        <v>378782</v>
+        <v>4462670</v>
       </c>
       <c r="G19" t="n">
-        <v>40</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1051</v>
+        <v>610</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="D20" t="n">
-        <v>0.5</v>
+        <v>4.8</v>
       </c>
       <c r="E20" t="n">
-        <v>6287249</v>
+        <v>10380012</v>
       </c>
       <c r="F20" t="n">
-        <v>2494800</v>
+        <v>4179980</v>
       </c>
       <c r="G20" t="n">
-        <v>39.7</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>146</v>
+        <v>1710</v>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="D21" t="n">
-        <v>6.8</v>
+        <v>4.6</v>
       </c>
       <c r="E21" t="n">
-        <v>5117175</v>
+        <v>37638384</v>
       </c>
       <c r="F21" t="n">
-        <v>1849190</v>
+        <v>13447508</v>
       </c>
       <c r="G21" t="n">
-        <v>36.1</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>323</v>
+        <v>3833</v>
       </c>
       <c r="C22" t="n">
-        <v>66</v>
+        <v>297</v>
       </c>
       <c r="D22" t="n">
-        <v>20.4</v>
+        <v>7.7</v>
       </c>
       <c r="E22" t="n">
-        <v>15079880</v>
+        <v>102510706</v>
       </c>
       <c r="F22" t="n">
-        <v>4594087</v>
+        <v>33516862</v>
       </c>
       <c r="G22" t="n">
-        <v>30.5</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3833</v>
+        <v>146</v>
       </c>
       <c r="C23" t="n">
-        <v>262</v>
+        <v>15</v>
       </c>
       <c r="D23" t="n">
-        <v>6.8</v>
+        <v>10.3</v>
       </c>
       <c r="E23" t="n">
-        <v>102510706</v>
+        <v>5117175</v>
       </c>
       <c r="F23" t="n">
-        <v>28387930</v>
+        <v>1379700</v>
       </c>
       <c r="G23" t="n">
-        <v>27.7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>272</v>
+        <v>3724</v>
       </c>
       <c r="C24" t="n">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="D24" t="n">
-        <v>2.9</v>
+        <v>1.7</v>
       </c>
       <c r="E24" t="n">
-        <v>4584179</v>
+        <v>71691344</v>
       </c>
       <c r="F24" t="n">
-        <v>1238712</v>
+        <v>19051684</v>
       </c>
       <c r="G24" t="n">
-        <v>27</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="25">
@@ -1050,69 +1050,69 @@
         <v>430</v>
       </c>
       <c r="C25" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D25" t="n">
-        <v>2.8</v>
+        <v>4.4</v>
       </c>
       <c r="E25" t="n">
         <v>10162018</v>
       </c>
       <c r="F25" t="n">
-        <v>2269960</v>
+        <v>2123000</v>
       </c>
       <c r="G25" t="n">
-        <v>22.3</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3724</v>
+        <v>272</v>
       </c>
       <c r="C26" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="D26" t="n">
-        <v>1.3</v>
+        <v>3.7</v>
       </c>
       <c r="E26" t="n">
-        <v>71691344</v>
+        <v>4584179</v>
       </c>
       <c r="F26" t="n">
-        <v>14375838</v>
+        <v>903354</v>
       </c>
       <c r="G26" t="n">
-        <v>20.1</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>117</v>
+        <v>72</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>1652034</v>
+        <v>1462612</v>
       </c>
       <c r="F27" t="n">
-        <v>259000</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>15.7</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>